<commit_message>
test: update XTB parser tests for account currency and PLN amounts
- Rewrite test expectations: currency from account header, amounts from Purchase/Sale value columns
- Add tests for detectAccountCurrency(), PLN pre-set rates, non-PLN accounts
- Regenerate fixture with realistic PLN amounts in Purchase/Sale value columns
- Add ticker extraction tests for exchange suffixes (.US, .UK, .DE)
- 50 tests covering all parser paths

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/src/__tests__/fixtures/xtb_closed_positions.xlsx
+++ b/src/__tests__/fixtures/xtb_closed_positions.xlsx
@@ -3,10 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="CLOSED POSITION HISTORY" sheetId="1" r:id="rId1"/>
-    <sheet name="OPEN POSITION 19042026" sheetId="2" r:id="rId2"/>
-    <sheet name="PENDING ORDERS HISTORY " sheetId="3" r:id="rId3"/>
-    <sheet name="CASH OPERATION HISTORY" sheetId="4" r:id="rId4"/>
+    <sheet name="CLOSED POSITION HISTORY " sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -401,25 +398,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X18"/>
+  <dimension ref="A1:U18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v/>
       </c>
-      <c r="L1" t="str">
+      <c r="B1" t="str">
         <v>History of transactions and operations</v>
       </c>
     </row>
     <row r="4">
-      <c r="E4" t="str">
+      <c r="A4" t="str">
         <v>Date range</v>
       </c>
-      <c r="H4" t="str">
+      <c r="B4" t="str">
         <v>2024-01-01 - 2025-12-31</v>
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="str">
+        <v/>
+      </c>
       <c r="B6" t="str">
         <v/>
       </c>
@@ -430,19 +430,19 @@
         <v/>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>Name and surname</v>
       </c>
       <c r="F6" t="str">
-        <v>Name and surname</v>
-      </c>
-      <c r="I6" t="str">
         <v>Account</v>
       </c>
-      <c r="L6" t="str">
+      <c r="G6" t="str">
         <v>Currency</v>
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
       <c r="B7" t="str">
         <v/>
       </c>
@@ -453,15 +453,12 @@
         <v/>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>Test User</v>
       </c>
       <c r="F7" t="str">
-        <v>Test User</v>
-      </c>
-      <c r="I7" t="str">
         <v>51723721</v>
       </c>
-      <c r="L7" t="str">
+      <c r="G7" t="str">
         <v>PLN</v>
       </c>
     </row>
@@ -469,8 +466,8 @@
       <c r="A12" t="str">
         <v/>
       </c>
-      <c r="U12" t="str">
-        <v>CLOSED POSITION HISTORY</v>
+      <c r="B12" t="str">
+        <v xml:space="preserve">CLOSED POSITION HISTORY </v>
       </c>
     </row>
     <row r="13">
@@ -555,13 +552,13 @@
         <v>2</v>
       </c>
       <c r="F14" s="1">
-        <v>45895.37505787037</v>
+        <v>45895.458391203705</v>
       </c>
       <c r="G14">
         <v>117.12</v>
       </c>
       <c r="H14" s="1">
-        <v>45966.37532407408</v>
+        <v>45966.41699074074</v>
       </c>
       <c r="I14">
         <v>118.1</v>
@@ -573,10 +570,10 @@
         <v>xStation 5</v>
       </c>
       <c r="L14">
-        <v>234.24</v>
+        <v>863.9</v>
       </c>
       <c r="M14">
-        <v>236.2</v>
+        <v>871.15</v>
       </c>
       <c r="Q14">
         <v>0</v>
@@ -590,9 +587,6 @@
       <c r="T14">
         <v>7.25</v>
       </c>
-      <c r="U14" t="str">
-        <v/>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -611,13 +605,13 @@
         <v>10</v>
       </c>
       <c r="F15" s="1">
-        <v>45672.416666666664</v>
+        <v>45672.458333333336</v>
       </c>
       <c r="G15">
         <v>185.5</v>
       </c>
       <c r="H15" s="1">
-        <v>45828.604166666664</v>
+        <v>45828.6875</v>
       </c>
       <c r="I15">
         <v>225.1</v>
@@ -629,10 +623,10 @@
         <v>xStation 5</v>
       </c>
       <c r="L15">
-        <v>1855</v>
+        <v>7500</v>
       </c>
       <c r="M15">
-        <v>2251</v>
+        <v>9000</v>
       </c>
       <c r="Q15">
         <v>0</v>
@@ -644,10 +638,7 @@
         <v>0</v>
       </c>
       <c r="T15">
-        <v>396</v>
-      </c>
-      <c r="U15" t="str">
-        <v/>
+        <v>1500</v>
       </c>
     </row>
     <row r="16">
@@ -667,13 +658,13 @@
         <v>5</v>
       </c>
       <c r="F16" s="1">
-        <v>45726.333333333336</v>
+        <v>45726.458333333336</v>
       </c>
       <c r="G16">
         <v>92.4</v>
       </c>
       <c r="H16" s="1">
-        <v>45915.5</v>
+        <v>45915.708333333336</v>
       </c>
       <c r="I16">
         <v>98.8</v>
@@ -685,10 +676,10 @@
         <v>xStation 5</v>
       </c>
       <c r="L16">
-        <v>462</v>
+        <v>2000</v>
       </c>
       <c r="M16">
-        <v>494</v>
+        <v>2150</v>
       </c>
       <c r="Q16">
         <v>0</v>
@@ -700,10 +691,7 @@
         <v>0</v>
       </c>
       <c r="T16">
-        <v>32</v>
-      </c>
-      <c r="U16" t="str">
-        <v/>
+        <v>150</v>
       </c>
     </row>
     <row r="17">
@@ -723,13 +711,13 @@
         <v>3</v>
       </c>
       <c r="F17" s="1">
-        <v>45301.375</v>
+        <v>45301.416666666664</v>
       </c>
       <c r="G17">
         <v>250</v>
       </c>
       <c r="H17" s="1">
-        <v>45473.625</v>
+        <v>45474.708333333336</v>
       </c>
       <c r="I17">
         <v>220</v>
@@ -741,10 +729,10 @@
         <v>xStation 5</v>
       </c>
       <c r="L17">
-        <v>750</v>
+        <v>3000</v>
       </c>
       <c r="M17">
-        <v>660</v>
+        <v>2640</v>
       </c>
       <c r="Q17">
         <v>0</v>
@@ -769,61 +757,22 @@
       <c r="B18" t="str">
         <v>Total</v>
       </c>
+      <c r="Q18">
+        <v>0</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+      <c r="S18">
+        <v>0</v>
+      </c>
       <c r="T18">
-        <v>335.25</v>
+        <v>1617.25</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X18"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Open positions</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Pending orders</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Cash operations</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>